<commit_message>
Daily EOD data and reports for 2026-10-22
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261022.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261022.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.68</v>
+        <v>1.677</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.005</v>
+        <v>-0.008</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>-0.47%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>257344.08</v>
+        <v>256884.54</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-765.91</v>
+        <v>-1225.45</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.405</v>
+        <v>2.415</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.005</v>
+        <v>0.015</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>168350</v>
+        <v>169050</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>350</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>57.48</v>
+        <v>57.31</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-1.06</v>
+        <v>-1.23</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-1.81%</t>
+          <t>-2.10%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>459840</v>
+        <v>458480</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-8480</v>
+        <v>-9840</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>156.84</v>
+        <v>157.4</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.17</v>
+        <v>0.39</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>0.25%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>194.99</v>
+        <v>195.81</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-1.09</v>
+        <v>-0.27</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>779960</v>
+        <v>783240</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-4360</v>
+        <v>-1080</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.205</v>
+        <v>0.2</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-2.44%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4100</v>
+        <v>4000</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11.42</v>
+        <v>11.45</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.03</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>34773.9</v>
+        <v>34865.25</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-91.34999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.081</v>
+        <v>0.08</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>762.37</v>
+        <v>752.96</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>9.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.415</v>
+        <v>35.55</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.115</v>
+        <v>0.02</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.77</v>
+        <v>32.775</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-1.19</v>
+        <v>-1.185</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.49%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42207.76</v>
+        <v>42214.2</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-1532.72</v>
+        <v>-1526.28</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1756088.56</v>
+        <v>1758237.4</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-16350.56</v>
+        <v>-14201.73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>